<commit_message>
agregar logica de envio y metodos asociados, correcion de setters para ordencompra y ordenenvio , se cambio el metodo __str__ de orden de compra
</commit_message>
<xml_diff>
--- a/inventario_televentas.xlsx
+++ b/inventario_televentas.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Productos" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Productos" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -706,7 +706,7 @@
         <v>150000</v>
       </c>
       <c r="E11" s="4" t="n">
-        <v>70</v>
+        <v>67</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
correcion actualizacion del stock en catalogo
</commit_message>
<xml_diff>
--- a/inventario_televentas.xlsx
+++ b/inventario_televentas.xlsx
@@ -545,7 +545,7 @@
         <v>260000</v>
       </c>
       <c r="E4" s="4" t="n">
-        <v>80</v>
+        <v>81</v>
       </c>
     </row>
     <row r="5">
@@ -568,7 +568,7 @@
         <v>1200000</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>25</v>
+        <v>22</v>
       </c>
     </row>
     <row r="6">
@@ -637,7 +637,7 @@
         <v>320000</v>
       </c>
       <c r="E8" s="4" t="n">
-        <v>90</v>
+        <v>92</v>
       </c>
     </row>
     <row r="9">
@@ -683,7 +683,7 @@
         <v>95000</v>
       </c>
       <c r="E10" s="4" t="n">
-        <v>200</v>
+        <v>199</v>
       </c>
     </row>
     <row r="11">
@@ -706,7 +706,7 @@
         <v>150000</v>
       </c>
       <c r="E11" s="4" t="n">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
   </sheetData>

</xml_diff>